<commit_message>
Update pipeline outputs for INFY, TCS, MARUTI, RELIANCE
- Refreshed cache JSON for INFY and RELIANCE
- Added MARUTI and TCS cache files
- Updated Excel reports for all 4 companies
- Added raw JSON outputs for all 4 companies

Co-Authored-By: Aakash Panchal & his team
</commit_message>
<xml_diff>
--- a/financial_analyzer/outputs/INFY_Financial_Analysis.xlsx
+++ b/financial_analyzer/outputs/INFY_Financial_Analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aakashpanchal/Desktop/Capstone Project/financial_analyzer/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99C07F1-77E3-484D-9F3F-0F4305A6CFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D65BD445A34C77A82F9CC83F26B2EDA54D700603" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -867,7 +867,7 @@
     <t xml:space="preserve">  Run Timestamp</t>
   </si>
   <si>
-    <t>2026-04-06 18:29:50</t>
+    <t>2026-04-08 21:24:24</t>
   </si>
   <si>
     <t xml:space="preserve">  Company Name</t>
@@ -1199,11 +1199,11 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.00\x"/>
     <numFmt numFmtId="166" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.0&quot;%&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.00\x;\(0.00\x\);&quot;-&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.0;\(0.0\);&quot;-&quot;"/>
-    <numFmt numFmtId="171" formatCode="&quot;-&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.00\x;\(0.00\x\);&quot;-&quot;"/>
+    <numFmt numFmtId="171" formatCode="0.0;\(0.0\);&quot;-&quot;"/>
+    <numFmt numFmtId="172" formatCode="&quot;-&quot;"/>
   </numFmts>
   <fonts count="41" x14ac:knownFonts="1">
     <font>
@@ -1631,7 +1631,7 @@
     <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1640,7 +1640,7 @@
     <xf numFmtId="166" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1653,10 +1653,10 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1665,10 +1665,10 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1678,13 +1678,13 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1693,13 +1693,13 @@
     <xf numFmtId="0" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1713,7 +1713,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="17" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1724,7 +1724,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1872,224 +1872,224 @@
     <xf numFmtId="0" fontId="9" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="38" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2406,7 +2406,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="134" t="s">
+      <c r="B2" s="112" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="95"/>
@@ -2424,7 +2424,7 @@
       <c r="O2" s="95"/>
     </row>
     <row r="3" spans="2:15" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="140" t="s">
+      <c r="B3" s="106" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="95"/>
@@ -2442,7 +2442,7 @@
       <c r="O3" s="95"/>
     </row>
     <row r="4" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="142" t="s">
+      <c r="B4" s="96" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="95"/>
@@ -2460,7 +2460,7 @@
       <c r="O4" s="95"/>
     </row>
     <row r="6" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="104" t="s">
+      <c r="B6" s="113" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="95"/>
@@ -2478,267 +2478,267 @@
       <c r="O6" s="95"/>
     </row>
     <row r="7" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="127" t="s">
+      <c r="B7" s="94" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="95"/>
       <c r="D7" s="95"/>
       <c r="E7" s="95"/>
       <c r="F7" s="95"/>
-      <c r="G7" s="127" t="s">
+      <c r="G7" s="94" t="s">
         <v>5</v>
       </c>
       <c r="H7" s="95"/>
       <c r="I7" s="95"/>
-      <c r="J7" s="127" t="s">
+      <c r="J7" s="94" t="s">
         <v>6</v>
       </c>
       <c r="K7" s="95"/>
-      <c r="L7" s="127" t="s">
+      <c r="L7" s="94" t="s">
         <v>7</v>
       </c>
       <c r="M7" s="95"/>
-      <c r="N7" s="127" t="s">
+      <c r="N7" s="94" t="s">
         <v>8</v>
       </c>
       <c r="O7" s="95"/>
     </row>
     <row r="8" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="131" t="s">
+      <c r="B8" s="100" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="95"/>
       <c r="D8" s="95"/>
       <c r="E8" s="95"/>
       <c r="F8" s="95"/>
-      <c r="G8" s="128" t="s">
+      <c r="G8" s="97" t="s">
         <v>10</v>
       </c>
       <c r="H8" s="95"/>
       <c r="I8" s="95"/>
-      <c r="J8" s="130">
+      <c r="J8" s="103">
         <v>6.0649443612936782E-2</v>
       </c>
       <c r="K8" s="95"/>
-      <c r="L8" s="137" t="s">
+      <c r="L8" s="102" t="s">
         <v>11</v>
       </c>
       <c r="M8" s="95"/>
-      <c r="N8" s="138" t="s">
+      <c r="N8" s="104" t="s">
         <v>12</v>
       </c>
       <c r="O8" s="95"/>
     </row>
     <row r="9" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="126" t="s">
+      <c r="B9" s="111" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="95"/>
       <c r="D9" s="95"/>
       <c r="E9" s="95"/>
       <c r="F9" s="95"/>
-      <c r="G9" s="132" t="s">
+      <c r="G9" s="99" t="s">
         <v>14</v>
       </c>
       <c r="H9" s="95"/>
       <c r="I9" s="95"/>
-      <c r="J9" s="139">
+      <c r="J9" s="110">
         <v>0.240726424934045</v>
       </c>
       <c r="K9" s="95"/>
-      <c r="L9" s="129" t="s">
+      <c r="L9" s="109" t="s">
         <v>15</v>
       </c>
       <c r="M9" s="95"/>
-      <c r="N9" s="125" t="s">
+      <c r="N9" s="98" t="s">
         <v>12</v>
       </c>
       <c r="O9" s="95"/>
     </row>
     <row r="10" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="131" t="s">
+      <c r="B10" s="100" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="95"/>
       <c r="D10" s="95"/>
       <c r="E10" s="95"/>
       <c r="F10" s="95"/>
-      <c r="G10" s="128" t="s">
+      <c r="G10" s="97" t="s">
         <v>14</v>
       </c>
       <c r="H10" s="95"/>
       <c r="I10" s="95"/>
-      <c r="J10" s="130">
+      <c r="J10" s="103">
         <v>0.16412049819007299</v>
       </c>
       <c r="K10" s="95"/>
-      <c r="L10" s="137" t="s">
+      <c r="L10" s="102" t="s">
         <v>17</v>
       </c>
       <c r="M10" s="95"/>
-      <c r="N10" s="138" t="s">
+      <c r="N10" s="104" t="s">
         <v>12</v>
       </c>
       <c r="O10" s="95"/>
     </row>
     <row r="11" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="126" t="s">
+      <c r="B11" s="111" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="95"/>
       <c r="D11" s="95"/>
       <c r="E11" s="95"/>
       <c r="F11" s="95"/>
-      <c r="G11" s="132" t="s">
+      <c r="G11" s="99" t="s">
         <v>19</v>
       </c>
       <c r="H11" s="95"/>
       <c r="I11" s="95"/>
-      <c r="J11" s="139">
+      <c r="J11" s="110">
         <v>0.29415645824627767</v>
       </c>
       <c r="K11" s="95"/>
-      <c r="L11" s="129" t="s">
+      <c r="L11" s="109" t="s">
         <v>20</v>
       </c>
       <c r="M11" s="95"/>
-      <c r="N11" s="125" t="s">
+      <c r="N11" s="98" t="s">
         <v>12</v>
       </c>
       <c r="O11" s="95"/>
     </row>
     <row r="12" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="131" t="s">
+      <c r="B12" s="100" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="95"/>
       <c r="D12" s="95"/>
       <c r="E12" s="95"/>
       <c r="F12" s="95"/>
-      <c r="G12" s="128" t="s">
+      <c r="G12" s="97" t="s">
         <v>19</v>
       </c>
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
-      <c r="J12" s="130">
+      <c r="J12" s="103">
         <v>0.34573401648474061</v>
       </c>
       <c r="K12" s="95"/>
-      <c r="L12" s="137" t="s">
+      <c r="L12" s="102" t="s">
         <v>22</v>
       </c>
       <c r="M12" s="95"/>
-      <c r="N12" s="138" t="s">
+      <c r="N12" s="104" t="s">
         <v>12</v>
       </c>
       <c r="O12" s="95"/>
     </row>
     <row r="13" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="126" t="s">
+      <c r="B13" s="111" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="95"/>
       <c r="D13" s="95"/>
       <c r="E13" s="95"/>
       <c r="F13" s="95"/>
-      <c r="G13" s="132" t="s">
+      <c r="G13" s="99" t="s">
         <v>24</v>
       </c>
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
-      <c r="J13" s="135">
+      <c r="J13" s="108">
         <v>0.98793625855683986</v>
       </c>
       <c r="K13" s="95"/>
-      <c r="L13" s="129" t="s">
+      <c r="L13" s="109" t="s">
         <v>25</v>
       </c>
       <c r="M13" s="95"/>
-      <c r="N13" s="133" t="s">
+      <c r="N13" s="114" t="s">
         <v>26</v>
       </c>
       <c r="O13" s="95"/>
     </row>
     <row r="14" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="131" t="s">
+      <c r="B14" s="100" t="s">
         <v>27</v>
       </c>
       <c r="C14" s="95"/>
       <c r="D14" s="95"/>
       <c r="E14" s="95"/>
       <c r="F14" s="95"/>
-      <c r="G14" s="128" t="s">
+      <c r="G14" s="97" t="s">
         <v>28</v>
       </c>
       <c r="H14" s="95"/>
       <c r="I14" s="95"/>
-      <c r="J14" s="141">
+      <c r="J14" s="101">
         <v>8.5484206151288447E-2</v>
       </c>
       <c r="K14" s="95"/>
-      <c r="L14" s="137" t="s">
+      <c r="L14" s="102" t="s">
         <v>29</v>
       </c>
       <c r="M14" s="95"/>
-      <c r="N14" s="138" t="s">
+      <c r="N14" s="104" t="s">
         <v>12</v>
       </c>
       <c r="O14" s="95"/>
     </row>
     <row r="15" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="126" t="s">
+      <c r="B15" s="111" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="95"/>
       <c r="D15" s="95"/>
       <c r="E15" s="95"/>
       <c r="F15" s="95"/>
-      <c r="G15" s="132" t="s">
+      <c r="G15" s="99" t="s">
         <v>28</v>
       </c>
       <c r="H15" s="95"/>
       <c r="I15" s="95"/>
-      <c r="J15" s="135">
+      <c r="J15" s="108">
         <v>91.40384615384616</v>
       </c>
       <c r="K15" s="95"/>
-      <c r="L15" s="129" t="s">
+      <c r="L15" s="109" t="s">
         <v>31</v>
       </c>
       <c r="M15" s="95"/>
-      <c r="N15" s="125" t="s">
+      <c r="N15" s="98" t="s">
         <v>12</v>
       </c>
       <c r="O15" s="95"/>
     </row>
     <row r="16" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="131" t="s">
+      <c r="B16" s="100" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="95"/>
       <c r="D16" s="95"/>
       <c r="E16" s="95"/>
       <c r="F16" s="95"/>
-      <c r="G16" s="128" t="s">
+      <c r="G16" s="97" t="s">
         <v>33</v>
       </c>
       <c r="H16" s="95"/>
       <c r="I16" s="95"/>
-      <c r="J16" s="130">
+      <c r="J16" s="103">
         <v>0.15370881649180931</v>
       </c>
       <c r="K16" s="95"/>
-      <c r="L16" s="137" t="s">
+      <c r="L16" s="102" t="s">
         <v>34</v>
       </c>
       <c r="M16" s="95"/>
-      <c r="N16" s="138" t="s">
+      <c r="N16" s="104" t="s">
         <v>12</v>
       </c>
       <c r="O16" s="95"/>
     </row>
     <row r="19" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="104" t="s">
+      <c r="B19" s="113" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="95"/>
@@ -2756,14 +2756,14 @@
       <c r="O19" s="95"/>
     </row>
     <row r="20" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="124" t="s">
+      <c r="B20" s="107" t="s">
         <v>36</v>
       </c>
       <c r="C20" s="95"/>
       <c r="D20" s="95"/>
       <c r="E20" s="95"/>
       <c r="F20" s="95"/>
-      <c r="G20" s="131" t="s">
+      <c r="G20" s="100" t="s">
         <v>37</v>
       </c>
       <c r="H20" s="95"/>
@@ -2776,14 +2776,14 @@
       <c r="O20" s="95"/>
     </row>
     <row r="21" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="136" t="s">
+      <c r="B21" s="105" t="s">
         <v>38</v>
       </c>
       <c r="C21" s="95"/>
       <c r="D21" s="95"/>
       <c r="E21" s="95"/>
       <c r="F21" s="95"/>
-      <c r="G21" s="126" t="s">
+      <c r="G21" s="111" t="s">
         <v>39</v>
       </c>
       <c r="H21" s="95"/>
@@ -2796,14 +2796,14 @@
       <c r="O21" s="95"/>
     </row>
     <row r="22" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="124" t="s">
+      <c r="B22" s="107" t="s">
         <v>40</v>
       </c>
       <c r="C22" s="95"/>
       <c r="D22" s="95"/>
       <c r="E22" s="95"/>
       <c r="F22" s="95"/>
-      <c r="G22" s="131" t="s">
+      <c r="G22" s="100" t="s">
         <v>41</v>
       </c>
       <c r="H22" s="95"/>
@@ -2816,14 +2816,14 @@
       <c r="O22" s="95"/>
     </row>
     <row r="23" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="136" t="s">
+      <c r="B23" s="105" t="s">
         <v>42</v>
       </c>
       <c r="C23" s="95"/>
       <c r="D23" s="95"/>
       <c r="E23" s="95"/>
       <c r="F23" s="95"/>
-      <c r="G23" s="126" t="s">
+      <c r="G23" s="111" t="s">
         <v>43</v>
       </c>
       <c r="H23" s="95"/>
@@ -2836,14 +2836,14 @@
       <c r="O23" s="95"/>
     </row>
     <row r="24" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="124" t="s">
+      <c r="B24" s="107" t="s">
         <v>44</v>
       </c>
       <c r="C24" s="95"/>
       <c r="D24" s="95"/>
       <c r="E24" s="95"/>
       <c r="F24" s="95"/>
-      <c r="G24" s="131" t="s">
+      <c r="G24" s="100" t="s">
         <v>45</v>
       </c>
       <c r="H24" s="95"/>
@@ -2856,14 +2856,14 @@
       <c r="O24" s="95"/>
     </row>
     <row r="25" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="136" t="s">
+      <c r="B25" s="105" t="s">
         <v>46</v>
       </c>
       <c r="C25" s="95"/>
       <c r="D25" s="95"/>
       <c r="E25" s="95"/>
       <c r="F25" s="95"/>
-      <c r="G25" s="126" t="s">
+      <c r="G25" s="111" t="s">
         <v>47</v>
       </c>
       <c r="H25" s="95"/>
@@ -2876,14 +2876,14 @@
       <c r="O25" s="95"/>
     </row>
     <row r="26" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="124" t="s">
+      <c r="B26" s="107" t="s">
         <v>48</v>
       </c>
       <c r="C26" s="95"/>
       <c r="D26" s="95"/>
       <c r="E26" s="95"/>
       <c r="F26" s="95"/>
-      <c r="G26" s="131" t="s">
+      <c r="G26" s="100" t="s">
         <v>49</v>
       </c>
       <c r="H26" s="95"/>
@@ -2897,49 +2897,11 @@
     </row>
   </sheetData>
   <mergeCells count="69">
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B4:O4"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="B3:O3"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="G20:O20"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B15:F15"/>
     <mergeCell ref="B6:O6"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="G23:O23"/>
@@ -2956,16 +2918,54 @@
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="N9:O9"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="G26:O26"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="G20:O20"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J11:K11"/>
     <mergeCell ref="G25:O25"/>
+    <mergeCell ref="N16:O16"/>
     <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="B21:F21"/>
     <mergeCell ref="G24:O24"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="J14:K14"/>
     <mergeCell ref="L16:M16"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B4:O4"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="N10:O10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2982,7 +2982,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="95"/>
@@ -2999,7 +2999,7 @@
       <c r="N2" s="95"/>
     </row>
     <row r="3" spans="2:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="115" t="s">
         <v>51</v>
       </c>
       <c r="C3" s="95"/>
@@ -3568,7 +3568,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>76</v>
       </c>
       <c r="C2" s="95"/>
@@ -3585,7 +3585,7 @@
       <c r="N2" s="95"/>
     </row>
     <row r="3" spans="2:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="115" t="s">
         <v>51</v>
       </c>
       <c r="C3" s="95"/>
@@ -4072,7 +4072,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>87</v>
       </c>
       <c r="C2" s="95"/>
@@ -4089,7 +4089,7 @@
       <c r="N2" s="95"/>
     </row>
     <row r="3" spans="2:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="115" t="s">
         <v>51</v>
       </c>
       <c r="C3" s="95"/>
@@ -5234,7 +5234,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>114</v>
       </c>
       <c r="C2" s="95"/>
@@ -6885,7 +6885,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="117" t="s">
         <v>148</v>
       </c>
       <c r="C2" s="95"/>
@@ -7279,7 +7279,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>158</v>
       </c>
       <c r="C2" s="95"/>
@@ -7296,7 +7296,7 @@
       <c r="N2" s="95"/>
     </row>
     <row r="3" spans="2:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="151" t="s">
+      <c r="B3" s="123" t="s">
         <v>159</v>
       </c>
       <c r="C3" s="95"/>
@@ -7313,7 +7313,7 @@
       <c r="N3" s="95"/>
     </row>
     <row r="5" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="104" t="s">
+      <c r="B5" s="113" t="s">
         <v>160</v>
       </c>
       <c r="C5" s="95"/>
@@ -7330,7 +7330,7 @@
       <c r="N5" s="95"/>
     </row>
     <row r="6" spans="2:14" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="154" t="s">
+      <c r="B6" s="121" t="s">
         <v>161</v>
       </c>
       <c r="C6" s="95"/>
@@ -7347,7 +7347,7 @@
       <c r="N6" s="95"/>
     </row>
     <row r="7" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="148" t="s">
+      <c r="B7" s="127" t="s">
         <v>162</v>
       </c>
       <c r="C7" s="95"/>
@@ -7417,7 +7417,7 @@
       </c>
     </row>
     <row r="13" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="150" t="s">
+      <c r="B13" s="119" t="s">
         <v>165</v>
       </c>
       <c r="C13" s="95"/>
@@ -7425,7 +7425,7 @@
       <c r="E13" s="95"/>
       <c r="F13" s="95"/>
       <c r="G13" s="95"/>
-      <c r="H13" s="149" t="s">
+      <c r="H13" s="118" t="s">
         <v>166</v>
       </c>
       <c r="I13" s="95"/>
@@ -7436,7 +7436,7 @@
       <c r="N13" s="95"/>
     </row>
     <row r="14" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="150" t="s">
+      <c r="B14" s="119" t="s">
         <v>167</v>
       </c>
       <c r="C14" s="95"/>
@@ -7444,7 +7444,7 @@
       <c r="E14" s="95"/>
       <c r="F14" s="95"/>
       <c r="G14" s="95"/>
-      <c r="H14" s="149" t="s">
+      <c r="H14" s="118" t="s">
         <v>168</v>
       </c>
       <c r="I14" s="95"/>
@@ -7455,7 +7455,7 @@
       <c r="N14" s="95"/>
     </row>
     <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="150" t="s">
+      <c r="B15" s="119" t="s">
         <v>169</v>
       </c>
       <c r="C15" s="95"/>
@@ -7463,7 +7463,7 @@
       <c r="E15" s="95"/>
       <c r="F15" s="95"/>
       <c r="G15" s="95"/>
-      <c r="H15" s="149" t="s">
+      <c r="H15" s="118" t="s">
         <v>170</v>
       </c>
       <c r="I15" s="95"/>
@@ -7474,7 +7474,7 @@
       <c r="N15" s="95"/>
     </row>
     <row r="17" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="104" t="s">
+      <c r="B17" s="113" t="s">
         <v>171</v>
       </c>
       <c r="C17" s="95"/>
@@ -7491,7 +7491,7 @@
       <c r="N17" s="95"/>
     </row>
     <row r="18" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="146" t="s">
+      <c r="B18" s="124" t="s">
         <v>172</v>
       </c>
       <c r="C18" s="95"/>
@@ -7508,7 +7508,7 @@
       <c r="N18" s="95"/>
     </row>
     <row r="19" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="147" t="s">
+      <c r="B19" s="122" t="s">
         <v>173</v>
       </c>
       <c r="C19" s="95"/>
@@ -7525,7 +7525,7 @@
       <c r="N19" s="95"/>
     </row>
     <row r="20" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="145" t="s">
+      <c r="B20" s="125" t="s">
         <v>174</v>
       </c>
       <c r="C20" s="95"/>
@@ -7557,7 +7557,7 @@
       <c r="N21" s="95"/>
     </row>
     <row r="23" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="146" t="s">
+      <c r="B23" s="124" t="s">
         <v>175</v>
       </c>
       <c r="C23" s="95"/>
@@ -7574,7 +7574,7 @@
       <c r="N23" s="95"/>
     </row>
     <row r="24" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="147" t="s">
+      <c r="B24" s="122" t="s">
         <v>176</v>
       </c>
       <c r="C24" s="95"/>
@@ -7591,7 +7591,7 @@
       <c r="N24" s="95"/>
     </row>
     <row r="25" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="145" t="s">
+      <c r="B25" s="125" t="s">
         <v>177</v>
       </c>
       <c r="C25" s="95"/>
@@ -7623,7 +7623,7 @@
       <c r="N26" s="95"/>
     </row>
     <row r="29" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="152" t="s">
+      <c r="B29" s="126" t="s">
         <v>178</v>
       </c>
       <c r="C29" s="95"/>
@@ -7640,7 +7640,7 @@
       <c r="N29" s="95"/>
     </row>
     <row r="30" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="153" t="s">
+      <c r="B30" s="120" t="s">
         <v>179</v>
       </c>
       <c r="C30" s="95"/>
@@ -7657,7 +7657,7 @@
       <c r="N30" s="95"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B32" s="150" t="s">
+      <c r="B32" s="119" t="s">
         <v>180</v>
       </c>
       <c r="C32" s="95"/>
@@ -7675,6 +7675,14 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B20:N21"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B19:N19"/>
+    <mergeCell ref="B7:N10"/>
+    <mergeCell ref="B5:N5"/>
+    <mergeCell ref="H14:N14"/>
     <mergeCell ref="B32:N32"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="B15:G15"/>
@@ -7688,14 +7696,6 @@
     <mergeCell ref="B6:N6"/>
     <mergeCell ref="B24:N24"/>
     <mergeCell ref="H15:N15"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B20:N21"/>
-    <mergeCell ref="B23:N23"/>
-    <mergeCell ref="B17:N17"/>
-    <mergeCell ref="B19:N19"/>
-    <mergeCell ref="B7:N10"/>
-    <mergeCell ref="B5:N5"/>
-    <mergeCell ref="H14:N14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7712,7 +7712,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="95"/>
@@ -7733,7 +7733,7 @@
       <c r="R2" s="95"/>
     </row>
     <row r="4" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="113" t="s">
         <v>182</v>
       </c>
       <c r="C4" s="95"/>
@@ -7812,7 +7812,7 @@
       </c>
     </row>
     <row r="10" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="104" t="s">
+      <c r="B10" s="113" t="s">
         <v>191</v>
       </c>
       <c r="C10" s="95"/>
@@ -8202,7 +8202,7 @@
       </c>
     </row>
     <row r="32" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="110" t="s">
+      <c r="B32" s="148" t="s">
         <v>212</v>
       </c>
       <c r="C32" s="95"/>
@@ -8592,7 +8592,7 @@
       </c>
     </row>
     <row r="54" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="111" t="s">
+      <c r="B54" s="151" t="s">
         <v>213</v>
       </c>
       <c r="C54" s="95"/>
@@ -8982,7 +8982,7 @@
       </c>
     </row>
     <row r="76" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="109" t="s">
+      <c r="B76" s="147" t="s">
         <v>214</v>
       </c>
       <c r="C76" s="95"/>
@@ -8995,74 +8995,74 @@
       <c r="J76" s="95"/>
     </row>
     <row r="77" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B77" s="98" t="s">
+      <c r="B77" s="134" t="s">
         <v>215</v>
       </c>
-      <c r="C77" s="97"/>
-      <c r="D77" s="96">
+      <c r="C77" s="129"/>
+      <c r="D77" s="137">
         <v>25053</v>
       </c>
-      <c r="E77" s="97"/>
+      <c r="E77" s="129"/>
     </row>
     <row r="78" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="98" t="s">
+      <c r="B78" s="134" t="s">
         <v>216</v>
       </c>
-      <c r="C78" s="97"/>
-      <c r="D78" s="96">
+      <c r="C78" s="129"/>
+      <c r="D78" s="137">
         <v>10.25</v>
       </c>
-      <c r="E78" s="97"/>
+      <c r="E78" s="129"/>
     </row>
     <row r="79" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="98" t="s">
+      <c r="B79" s="134" t="s">
         <v>217</v>
       </c>
-      <c r="C79" s="97"/>
-      <c r="D79" s="96">
+      <c r="C79" s="129"/>
+      <c r="D79" s="137">
         <v>9.8245360574943685</v>
       </c>
-      <c r="E79" s="97"/>
+      <c r="E79" s="129"/>
     </row>
     <row r="80" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B80" s="98" t="s">
+      <c r="B80" s="134" t="s">
         <v>218</v>
       </c>
-      <c r="C80" s="97"/>
-      <c r="D80" s="96">
+      <c r="C80" s="129"/>
+      <c r="D80" s="137">
         <v>4</v>
       </c>
-      <c r="E80" s="97"/>
+      <c r="E80" s="129"/>
     </row>
     <row r="81" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B81" s="98" t="s">
+      <c r="B81" s="134" t="s">
         <v>219</v>
       </c>
-      <c r="C81" s="97"/>
-      <c r="D81" s="96">
+      <c r="C81" s="129"/>
+      <c r="D81" s="137">
         <v>5</v>
       </c>
-      <c r="E81" s="97"/>
+      <c r="E81" s="129"/>
     </row>
     <row r="82" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="98" t="s">
+      <c r="B82" s="134" t="s">
         <v>136</v>
       </c>
-      <c r="C82" s="97"/>
-      <c r="D82" s="96">
+      <c r="C82" s="129"/>
+      <c r="D82" s="137">
         <v>-11007</v>
       </c>
-      <c r="E82" s="97"/>
+      <c r="E82" s="129"/>
     </row>
     <row r="83" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="98" t="s">
+      <c r="B83" s="134" t="s">
         <v>220</v>
       </c>
-      <c r="C83" s="97"/>
-      <c r="D83" s="96">
+      <c r="C83" s="129"/>
+      <c r="D83" s="137">
         <v>5</v>
       </c>
-      <c r="E83" s="97"/>
+      <c r="E83" s="129"/>
     </row>
     <row r="85" spans="2:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B85" s="1" t="s">
@@ -9131,67 +9131,67 @@
       </c>
     </row>
     <row r="92" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="99" t="s">
+      <c r="B92" s="138" t="s">
         <v>224</v>
       </c>
-      <c r="C92" s="97"/>
-      <c r="D92" s="105">
+      <c r="C92" s="129"/>
+      <c r="D92" s="140">
         <v>728506</v>
       </c>
-      <c r="E92" s="97"/>
+      <c r="E92" s="129"/>
     </row>
     <row r="93" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="99" t="s">
+      <c r="B93" s="138" t="s">
         <v>225</v>
       </c>
-      <c r="C93" s="97"/>
-      <c r="D93" s="105">
+      <c r="C93" s="129"/>
+      <c r="D93" s="140">
         <v>455970</v>
       </c>
-      <c r="E93" s="97"/>
+      <c r="E93" s="129"/>
     </row>
     <row r="94" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="99" t="s">
+      <c r="B94" s="138" t="s">
         <v>226</v>
       </c>
-      <c r="C94" s="97"/>
-      <c r="D94" s="105">
+      <c r="C94" s="129"/>
+      <c r="D94" s="140">
         <v>582682</v>
       </c>
-      <c r="E94" s="97"/>
+      <c r="E94" s="129"/>
     </row>
     <row r="95" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="99" t="s">
+      <c r="B95" s="138" t="s">
         <v>136</v>
       </c>
-      <c r="C95" s="97"/>
-      <c r="D95" s="105">
+      <c r="C95" s="129"/>
+      <c r="D95" s="140">
         <v>-11007</v>
       </c>
-      <c r="E95" s="97"/>
+      <c r="E95" s="129"/>
     </row>
     <row r="96" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B96" s="99" t="s">
+      <c r="B96" s="138" t="s">
         <v>227</v>
       </c>
-      <c r="C96" s="97"/>
-      <c r="D96" s="105">
+      <c r="C96" s="129"/>
+      <c r="D96" s="140">
         <v>593689</v>
       </c>
-      <c r="E96" s="97"/>
+      <c r="E96" s="129"/>
     </row>
     <row r="97" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B97" s="121" t="s">
+      <c r="B97" s="128" t="s">
         <v>228</v>
       </c>
-      <c r="C97" s="97"/>
-      <c r="D97" s="108">
+      <c r="C97" s="129"/>
+      <c r="D97" s="143">
         <v>1432</v>
       </c>
-      <c r="E97" s="97"/>
+      <c r="E97" s="129"/>
     </row>
     <row r="99" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="106" t="s">
+      <c r="B99" s="142" t="s">
         <v>229</v>
       </c>
       <c r="C99" s="95"/>
@@ -9204,7 +9204,7 @@
       <c r="J99" s="95"/>
     </row>
     <row r="100" spans="2:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="117" t="s">
+      <c r="B100" s="150" t="s">
         <v>230</v>
       </c>
       <c r="C100" s="95"/>
@@ -9217,19 +9217,19 @@
       <c r="J100" s="95"/>
     </row>
     <row r="102" spans="2:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B102" s="114" t="s">
+      <c r="B102" s="144" t="s">
         <v>231</v>
       </c>
       <c r="C102" s="95"/>
       <c r="D102" s="95"/>
       <c r="E102" s="95"/>
-      <c r="F102" s="122" t="s">
+      <c r="F102" s="131" t="s">
         <v>232</v>
       </c>
       <c r="G102" s="95"/>
       <c r="H102" s="95"/>
       <c r="I102" s="95"/>
-      <c r="J102" s="115" t="s">
+      <c r="J102" s="145" t="s">
         <v>233</v>
       </c>
       <c r="K102" s="95"/>
@@ -9237,19 +9237,19 @@
       <c r="M102" s="95"/>
     </row>
     <row r="103" spans="2:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B103" s="101" t="s">
+      <c r="B103" s="146" t="s">
         <v>234</v>
       </c>
       <c r="C103" s="95"/>
       <c r="D103" s="95"/>
       <c r="E103" s="95"/>
-      <c r="F103" s="113" t="s">
+      <c r="F103" s="132" t="s">
         <v>235</v>
       </c>
       <c r="G103" s="95"/>
       <c r="H103" s="95"/>
       <c r="I103" s="95"/>
-      <c r="J103" s="102" t="s">
+      <c r="J103" s="136" t="s">
         <v>236</v>
       </c>
       <c r="K103" s="95"/>
@@ -9257,19 +9257,19 @@
       <c r="M103" s="95"/>
     </row>
     <row r="104" spans="2:13" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B104" s="120" t="s">
+      <c r="B104" s="139" t="s">
         <v>237</v>
       </c>
       <c r="C104" s="95"/>
       <c r="D104" s="95"/>
       <c r="E104" s="95"/>
-      <c r="F104" s="116" t="s">
+      <c r="F104" s="149" t="s">
         <v>238</v>
       </c>
       <c r="G104" s="95"/>
       <c r="H104" s="95"/>
       <c r="I104" s="95"/>
-      <c r="J104" s="100" t="s">
+      <c r="J104" s="153" t="s">
         <v>239</v>
       </c>
       <c r="K104" s="95"/>
@@ -9277,19 +9277,19 @@
       <c r="M104" s="95"/>
     </row>
     <row r="105" spans="2:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B105" s="101" t="s">
+      <c r="B105" s="146" t="s">
         <v>240</v>
       </c>
       <c r="C105" s="95"/>
       <c r="D105" s="95"/>
       <c r="E105" s="95"/>
-      <c r="F105" s="113" t="s">
+      <c r="F105" s="132" t="s">
         <v>241</v>
       </c>
       <c r="G105" s="95"/>
       <c r="H105" s="95"/>
       <c r="I105" s="95"/>
-      <c r="J105" s="102" t="s">
+      <c r="J105" s="136" t="s">
         <v>242</v>
       </c>
       <c r="K105" s="95"/>
@@ -9297,7 +9297,7 @@
       <c r="M105" s="95"/>
     </row>
     <row r="107" spans="2:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B107" s="123" t="s">
+      <c r="B107" s="133" t="s">
         <v>243</v>
       </c>
       <c r="C107" s="95"/>
@@ -9310,7 +9310,7 @@
       <c r="J107" s="95"/>
     </row>
     <row r="109" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B109" s="118" t="s">
+      <c r="B109" s="135" t="s">
         <v>244</v>
       </c>
       <c r="C109" s="95"/>
@@ -9525,7 +9525,7 @@
       </c>
     </row>
     <row r="122" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B122" s="112" t="s">
+      <c r="B122" s="141" t="s">
         <v>260</v>
       </c>
       <c r="C122" s="95"/>
@@ -9546,7 +9546,7 @@
       <c r="R122" s="95"/>
     </row>
     <row r="123" spans="2:19" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B123" s="103" t="s">
+      <c r="B123" s="154" t="s">
         <v>261</v>
       </c>
       <c r="C123" s="95"/>
@@ -9567,7 +9567,7 @@
       <c r="R123" s="95"/>
     </row>
     <row r="124" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B124" s="119" t="s">
+      <c r="B124" s="130" t="s">
         <v>262</v>
       </c>
       <c r="C124" s="95"/>
@@ -9741,19 +9741,19 @@
         <v>162990</v>
       </c>
       <c r="O127" s="71">
-        <v>174593</v>
+        <v>174992</v>
       </c>
       <c r="P127" s="71">
-        <v>189469</v>
+        <v>189314</v>
       </c>
       <c r="Q127" s="71">
-        <v>203186</v>
+        <v>203242</v>
       </c>
       <c r="R127" s="71">
-        <v>216427</v>
+        <v>216250</v>
       </c>
       <c r="S127" s="71">
-        <v>229458</v>
+        <v>228659</v>
       </c>
     </row>
     <row r="128" spans="2:19" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -9797,23 +9797,23 @@
         <v>162990</v>
       </c>
       <c r="O128" s="73">
-        <v>184383</v>
+        <v>184501</v>
       </c>
       <c r="P128" s="73">
-        <v>200163</v>
+        <v>200588</v>
       </c>
       <c r="Q128" s="73">
-        <v>216975</v>
+        <v>216817</v>
       </c>
       <c r="R128" s="73">
-        <v>233914</v>
+        <v>234844</v>
       </c>
       <c r="S128" s="73">
-        <v>252609</v>
+        <v>252532</v>
       </c>
     </row>
     <row r="130" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B130" s="119" t="s">
+      <c r="B130" s="130" t="s">
         <v>267</v>
       </c>
       <c r="C130" s="95"/>
@@ -9987,19 +9987,19 @@
         <v>39236</v>
       </c>
       <c r="O133" s="71">
-        <v>40365</v>
+        <v>40257</v>
       </c>
       <c r="P133" s="71">
-        <v>41137</v>
+        <v>41383</v>
       </c>
       <c r="Q133" s="71">
-        <v>41574</v>
+        <v>41538</v>
       </c>
       <c r="R133" s="71">
-        <v>41318</v>
+        <v>41315</v>
       </c>
       <c r="S133" s="71">
-        <v>40993</v>
+        <v>41280</v>
       </c>
     </row>
     <row r="134" spans="2:19" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -10043,23 +10043,23 @@
         <v>39236</v>
       </c>
       <c r="O134" s="73">
-        <v>41982</v>
+        <v>41928</v>
       </c>
       <c r="P134" s="73">
-        <v>45841</v>
+        <v>45866</v>
       </c>
       <c r="Q134" s="73">
-        <v>50387</v>
+        <v>50705</v>
       </c>
       <c r="R134" s="73">
-        <v>55469</v>
+        <v>55399</v>
       </c>
       <c r="S134" s="73">
-        <v>61233</v>
+        <v>61052</v>
       </c>
     </row>
     <row r="136" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B136" s="119" t="s">
+      <c r="B136" s="130" t="s">
         <v>140</v>
       </c>
       <c r="C136" s="95"/>
@@ -10233,19 +10233,19 @@
         <v>25053</v>
       </c>
       <c r="O139" s="71">
-        <v>19940</v>
+        <v>19705</v>
       </c>
       <c r="P139" s="71">
-        <v>21696</v>
+        <v>21528</v>
       </c>
       <c r="Q139" s="71">
-        <v>23014</v>
+        <v>23470</v>
       </c>
       <c r="R139" s="71">
-        <v>24631</v>
+        <v>24959</v>
       </c>
       <c r="S139" s="71">
-        <v>26151</v>
+        <v>26534</v>
       </c>
     </row>
     <row r="140" spans="2:19" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -10289,23 +10289,23 @@
         <v>25053</v>
       </c>
       <c r="O140" s="73">
-        <v>26926</v>
+        <v>26713</v>
       </c>
       <c r="P140" s="73">
-        <v>28351</v>
+        <v>28599</v>
       </c>
       <c r="Q140" s="73">
-        <v>30116</v>
+        <v>29861</v>
       </c>
       <c r="R140" s="73">
-        <v>31805</v>
+        <v>31738</v>
       </c>
       <c r="S140" s="73">
-        <v>33168</v>
+        <v>33346</v>
       </c>
     </row>
     <row r="143" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B143" s="94" t="s">
+      <c r="B143" s="152" t="s">
         <v>268</v>
       </c>
       <c r="C143" s="95"/>
@@ -10431,19 +10431,19 @@
         <v>274</v>
       </c>
       <c r="C150" s="84">
-        <v>184383</v>
+        <v>184501</v>
       </c>
       <c r="D150" s="84">
-        <v>200163</v>
+        <v>200588</v>
       </c>
       <c r="E150" s="84">
-        <v>216975</v>
+        <v>216817</v>
       </c>
       <c r="F150" s="84">
-        <v>233914</v>
+        <v>234844</v>
       </c>
       <c r="G150" s="84">
-        <v>252609</v>
+        <v>252532</v>
       </c>
     </row>
     <row r="151" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10451,19 +10451,19 @@
         <v>275</v>
       </c>
       <c r="C151" s="86">
-        <v>174593</v>
+        <v>174992</v>
       </c>
       <c r="D151" s="86">
-        <v>189469</v>
+        <v>189314</v>
       </c>
       <c r="E151" s="86">
-        <v>203186</v>
+        <v>203242</v>
       </c>
       <c r="F151" s="86">
-        <v>216427</v>
+        <v>216250</v>
       </c>
       <c r="G151" s="86">
-        <v>229458</v>
+        <v>228659</v>
       </c>
     </row>
     <row r="152" spans="2:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -10488,28 +10488,15 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="J105:M105"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="B136:S136"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="B124:S124"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B130:S130"/>
-    <mergeCell ref="F102:I102"/>
-    <mergeCell ref="F105:I105"/>
-    <mergeCell ref="B107:J107"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="F103:I103"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="J102:M102"/>
-    <mergeCell ref="B100:J100"/>
-    <mergeCell ref="D92:E92"/>
-    <mergeCell ref="D94:E94"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="D79:E79"/>
-    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B143:R143"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="J104:M104"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="J103:M103"/>
+    <mergeCell ref="B123:R123"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="D95:E95"/>
     <mergeCell ref="B4:H4"/>
@@ -10526,22 +10513,35 @@
     <mergeCell ref="D83:E83"/>
     <mergeCell ref="B54:G54"/>
     <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B143:R143"/>
-    <mergeCell ref="D82:E82"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="J104:M104"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="J103:M103"/>
-    <mergeCell ref="B123:R123"/>
     <mergeCell ref="D80:E80"/>
     <mergeCell ref="B96:C96"/>
     <mergeCell ref="D96:E96"/>
     <mergeCell ref="B122:R122"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="F103:I103"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="J102:M102"/>
     <mergeCell ref="B105:E105"/>
     <mergeCell ref="F104:I104"/>
+    <mergeCell ref="B100:J100"/>
+    <mergeCell ref="D92:E92"/>
+    <mergeCell ref="D94:E94"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="B81:C81"/>
     <mergeCell ref="B109:L109"/>
+    <mergeCell ref="J105:M105"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="B136:S136"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B104:E104"/>
+    <mergeCell ref="B124:S124"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B130:S130"/>
+    <mergeCell ref="F102:I102"/>
+    <mergeCell ref="F105:I105"/>
+    <mergeCell ref="B107:J107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10555,11 +10555,10 @@
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="116" t="s">
         <v>277</v>
       </c>
       <c r="C2" s="95"/>
@@ -10570,176 +10569,176 @@
       <c r="H2" s="95"/>
     </row>
     <row r="4" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="158" t="s">
+      <c r="B4" s="166" t="s">
         <v>278</v>
       </c>
       <c r="C4" s="156"/>
-      <c r="D4" s="97"/>
-      <c r="E4" s="170" t="s">
+      <c r="D4" s="129"/>
+      <c r="E4" s="167" t="s">
         <v>279</v>
       </c>
       <c r="F4" s="156"/>
       <c r="G4" s="156"/>
-      <c r="H4" s="97"/>
+      <c r="H4" s="129"/>
     </row>
     <row r="5" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="155" t="s">
         <v>280</v>
       </c>
       <c r="C5" s="156"/>
-      <c r="D5" s="97"/>
-      <c r="E5" s="98" t="s">
+      <c r="D5" s="129"/>
+      <c r="E5" s="134" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="156"/>
       <c r="G5" s="156"/>
-      <c r="H5" s="97"/>
+      <c r="H5" s="129"/>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="158" t="s">
+      <c r="B6" s="166" t="s">
         <v>281</v>
       </c>
       <c r="C6" s="156"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="170" t="s">
+      <c r="D6" s="129"/>
+      <c r="E6" s="167" t="s">
         <v>1</v>
       </c>
       <c r="F6" s="156"/>
       <c r="G6" s="156"/>
-      <c r="H6" s="97"/>
+      <c r="H6" s="129"/>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="155" t="s">
         <v>282</v>
       </c>
       <c r="C7" s="156"/>
-      <c r="D7" s="97"/>
-      <c r="E7" s="98" t="s">
+      <c r="D7" s="129"/>
+      <c r="E7" s="134" t="s">
         <v>283</v>
       </c>
       <c r="F7" s="156"/>
       <c r="G7" s="156"/>
-      <c r="H7" s="97"/>
+      <c r="H7" s="129"/>
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="158" t="s">
+      <c r="B8" s="166" t="s">
         <v>284</v>
       </c>
       <c r="C8" s="156"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="170" t="s">
+      <c r="D8" s="129"/>
+      <c r="E8" s="167" t="s">
         <v>285</v>
       </c>
       <c r="F8" s="156"/>
       <c r="G8" s="156"/>
-      <c r="H8" s="97"/>
+      <c r="H8" s="129"/>
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="155" t="s">
         <v>286</v>
       </c>
       <c r="C9" s="156"/>
-      <c r="D9" s="97"/>
-      <c r="E9" s="98" t="s">
+      <c r="D9" s="129"/>
+      <c r="E9" s="134" t="s">
         <v>287</v>
       </c>
       <c r="F9" s="156"/>
       <c r="G9" s="156"/>
-      <c r="H9" s="97"/>
+      <c r="H9" s="129"/>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="158" t="s">
+      <c r="B10" s="166" t="s">
         <v>288</v>
       </c>
       <c r="C10" s="156"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="170" t="s">
+      <c r="D10" s="129"/>
+      <c r="E10" s="167" t="s">
         <v>289</v>
       </c>
       <c r="F10" s="156"/>
       <c r="G10" s="156"/>
-      <c r="H10" s="97"/>
+      <c r="H10" s="129"/>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="155" t="s">
         <v>290</v>
       </c>
       <c r="C11" s="156"/>
-      <c r="D11" s="97"/>
-      <c r="E11" s="98" t="s">
+      <c r="D11" s="129"/>
+      <c r="E11" s="134" t="s">
         <v>291</v>
       </c>
       <c r="F11" s="156"/>
       <c r="G11" s="156"/>
-      <c r="H11" s="97"/>
+      <c r="H11" s="129"/>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="158" t="s">
+      <c r="B12" s="166" t="s">
         <v>292</v>
       </c>
       <c r="C12" s="156"/>
-      <c r="D12" s="97"/>
-      <c r="E12" s="170" t="s">
+      <c r="D12" s="129"/>
+      <c r="E12" s="167" t="s">
         <v>293</v>
       </c>
       <c r="F12" s="156"/>
       <c r="G12" s="156"/>
-      <c r="H12" s="97"/>
+      <c r="H12" s="129"/>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="155" t="s">
         <v>294</v>
       </c>
       <c r="C13" s="156"/>
-      <c r="D13" s="97"/>
-      <c r="E13" s="98" t="s">
+      <c r="D13" s="129"/>
+      <c r="E13" s="134" t="s">
         <v>295</v>
       </c>
       <c r="F13" s="156"/>
       <c r="G13" s="156"/>
-      <c r="H13" s="97"/>
+      <c r="H13" s="129"/>
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="158" t="s">
+      <c r="B14" s="166" t="s">
         <v>296</v>
       </c>
       <c r="C14" s="156"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="170" t="s">
+      <c r="D14" s="129"/>
+      <c r="E14" s="167" t="s">
         <v>297</v>
       </c>
       <c r="F14" s="156"/>
       <c r="G14" s="156"/>
-      <c r="H14" s="97"/>
+      <c r="H14" s="129"/>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="155" t="s">
         <v>298</v>
       </c>
       <c r="C15" s="156"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="98" t="s">
+      <c r="D15" s="129"/>
+      <c r="E15" s="134" t="s">
         <v>299</v>
       </c>
       <c r="F15" s="156"/>
       <c r="G15" s="156"/>
-      <c r="H15" s="97"/>
+      <c r="H15" s="129"/>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="158" t="s">
+      <c r="B16" s="166" t="s">
         <v>300</v>
       </c>
       <c r="C16" s="156"/>
-      <c r="D16" s="97"/>
-      <c r="E16" s="170" t="s">
+      <c r="D16" s="129"/>
+      <c r="E16" s="167" t="s">
         <v>301</v>
       </c>
       <c r="F16" s="156"/>
       <c r="G16" s="156"/>
-      <c r="H16" s="97"/>
+      <c r="H16" s="129"/>
     </row>
     <row r="19" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="104" t="s">
+      <c r="B19" s="113" t="s">
         <v>302</v>
       </c>
       <c r="C19" s="95"/>
@@ -10756,7 +10755,7 @@
       <c r="N19" s="95"/>
     </row>
     <row r="20" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="131" t="s">
+      <c r="B20" s="100" t="s">
         <v>303</v>
       </c>
       <c r="C20" s="95"/>
@@ -10775,26 +10774,26 @@
       <c r="N20" s="95"/>
     </row>
     <row r="21" spans="2:14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="168" t="s">
+      <c r="B21" s="164" t="s">
         <v>305</v>
       </c>
       <c r="C21" s="95"/>
-      <c r="D21" s="168" t="s">
+      <c r="D21" s="164" t="s">
         <v>269</v>
       </c>
       <c r="E21" s="95"/>
-      <c r="F21" s="168" t="s">
+      <c r="F21" s="164" t="s">
         <v>306</v>
       </c>
       <c r="G21" s="95"/>
-      <c r="H21" s="168" t="s">
+      <c r="H21" s="164" t="s">
         <v>307</v>
       </c>
       <c r="I21" s="95"/>
       <c r="J21" s="90" t="s">
         <v>308</v>
       </c>
-      <c r="K21" s="168" t="s">
+      <c r="K21" s="164" t="s">
         <v>309</v>
       </c>
       <c r="L21" s="95"/>
@@ -10802,26 +10801,26 @@
       <c r="N21" s="95"/>
     </row>
     <row r="22" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="164" t="s">
+      <c r="B22" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C22" s="95"/>
-      <c r="D22" s="159" t="s">
+      <c r="D22" s="162" t="s">
         <v>311</v>
       </c>
       <c r="E22" s="95"/>
-      <c r="F22" s="159" t="s">
+      <c r="F22" s="162" t="s">
         <v>312</v>
       </c>
       <c r="G22" s="95"/>
-      <c r="H22" s="159" t="s">
+      <c r="H22" s="162" t="s">
         <v>313</v>
       </c>
       <c r="I22" s="95"/>
       <c r="J22" s="91" t="s">
         <v>314</v>
       </c>
-      <c r="K22" s="159" t="s">
+      <c r="K22" s="162" t="s">
         <v>315</v>
       </c>
       <c r="L22" s="95"/>
@@ -10829,26 +10828,26 @@
       <c r="N22" s="95"/>
     </row>
     <row r="23" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="169" t="s">
+      <c r="B23" s="171" t="s">
         <v>316</v>
       </c>
       <c r="C23" s="95"/>
-      <c r="D23" s="166" t="s">
+      <c r="D23" s="168" t="s">
         <v>311</v>
       </c>
       <c r="E23" s="95"/>
-      <c r="F23" s="166" t="s">
+      <c r="F23" s="168" t="s">
         <v>317</v>
       </c>
       <c r="G23" s="95"/>
-      <c r="H23" s="166" t="s">
+      <c r="H23" s="168" t="s">
         <v>318</v>
       </c>
       <c r="I23" s="95"/>
       <c r="J23" s="92" t="s">
         <v>319</v>
       </c>
-      <c r="K23" s="166" t="s">
+      <c r="K23" s="168" t="s">
         <v>320</v>
       </c>
       <c r="L23" s="95"/>
@@ -10856,26 +10855,26 @@
       <c r="N23" s="95"/>
     </row>
     <row r="24" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="164" t="s">
+      <c r="B24" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C24" s="95"/>
-      <c r="D24" s="159" t="s">
+      <c r="D24" s="162" t="s">
         <v>311</v>
       </c>
       <c r="E24" s="95"/>
-      <c r="F24" s="159" t="s">
+      <c r="F24" s="162" t="s">
         <v>321</v>
       </c>
       <c r="G24" s="95"/>
-      <c r="H24" s="159" t="s">
+      <c r="H24" s="162" t="s">
         <v>322</v>
       </c>
       <c r="I24" s="95"/>
       <c r="J24" s="91" t="s">
         <v>323</v>
       </c>
-      <c r="K24" s="159" t="s">
+      <c r="K24" s="162" t="s">
         <v>324</v>
       </c>
       <c r="L24" s="95"/>
@@ -10883,26 +10882,26 @@
       <c r="N24" s="95"/>
     </row>
     <row r="25" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="171" t="s">
+      <c r="B25" s="163" t="s">
         <v>310</v>
       </c>
       <c r="C25" s="95"/>
-      <c r="D25" s="157" t="s">
+      <c r="D25" s="158" t="s">
         <v>311</v>
       </c>
       <c r="E25" s="95"/>
-      <c r="F25" s="157" t="s">
+      <c r="F25" s="158" t="s">
         <v>325</v>
       </c>
       <c r="G25" s="95"/>
-      <c r="H25" s="157" t="s">
+      <c r="H25" s="158" t="s">
         <v>322</v>
       </c>
       <c r="I25" s="95"/>
       <c r="J25" s="93" t="s">
         <v>326</v>
       </c>
-      <c r="K25" s="157" t="s">
+      <c r="K25" s="158" t="s">
         <v>327</v>
       </c>
       <c r="L25" s="95"/>
@@ -10910,26 +10909,26 @@
       <c r="N25" s="95"/>
     </row>
     <row r="26" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="164" t="s">
+      <c r="B26" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C26" s="95"/>
-      <c r="D26" s="159" t="s">
+      <c r="D26" s="162" t="s">
         <v>311</v>
       </c>
       <c r="E26" s="95"/>
-      <c r="F26" s="159" t="s">
+      <c r="F26" s="162" t="s">
         <v>328</v>
       </c>
       <c r="G26" s="95"/>
-      <c r="H26" s="159" t="s">
+      <c r="H26" s="162" t="s">
         <v>322</v>
       </c>
       <c r="I26" s="95"/>
       <c r="J26" s="91" t="s">
         <v>329</v>
       </c>
-      <c r="K26" s="159" t="s">
+      <c r="K26" s="162" t="s">
         <v>330</v>
       </c>
       <c r="L26" s="95"/>
@@ -10937,26 +10936,26 @@
       <c r="N26" s="95"/>
     </row>
     <row r="27" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="171" t="s">
+      <c r="B27" s="163" t="s">
         <v>310</v>
       </c>
       <c r="C27" s="95"/>
-      <c r="D27" s="157" t="s">
+      <c r="D27" s="158" t="s">
         <v>311</v>
       </c>
       <c r="E27" s="95"/>
-      <c r="F27" s="157" t="s">
+      <c r="F27" s="158" t="s">
         <v>331</v>
       </c>
       <c r="G27" s="95"/>
-      <c r="H27" s="157" t="s">
+      <c r="H27" s="158" t="s">
         <v>322</v>
       </c>
       <c r="I27" s="95"/>
       <c r="J27" s="93" t="s">
         <v>332</v>
       </c>
-      <c r="K27" s="157" t="s">
+      <c r="K27" s="158" t="s">
         <v>333</v>
       </c>
       <c r="L27" s="95"/>
@@ -10964,26 +10963,26 @@
       <c r="N27" s="95"/>
     </row>
     <row r="28" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="164" t="s">
+      <c r="B28" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C28" s="95"/>
-      <c r="D28" s="159" t="s">
+      <c r="D28" s="162" t="s">
         <v>311</v>
       </c>
       <c r="E28" s="95"/>
-      <c r="F28" s="159" t="s">
+      <c r="F28" s="162" t="s">
         <v>334</v>
       </c>
       <c r="G28" s="95"/>
-      <c r="H28" s="159" t="s">
+      <c r="H28" s="162" t="s">
         <v>322</v>
       </c>
       <c r="I28" s="95"/>
       <c r="J28" s="91" t="s">
         <v>335</v>
       </c>
-      <c r="K28" s="159" t="s">
+      <c r="K28" s="162" t="s">
         <v>336</v>
       </c>
       <c r="L28" s="95"/>
@@ -10991,26 +10990,26 @@
       <c r="N28" s="95"/>
     </row>
     <row r="29" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="171" t="s">
+      <c r="B29" s="163" t="s">
         <v>310</v>
       </c>
       <c r="C29" s="95"/>
-      <c r="D29" s="157" t="s">
+      <c r="D29" s="158" t="s">
         <v>311</v>
       </c>
       <c r="E29" s="95"/>
-      <c r="F29" s="157" t="s">
+      <c r="F29" s="158" t="s">
         <v>337</v>
       </c>
       <c r="G29" s="95"/>
-      <c r="H29" s="157" t="s">
+      <c r="H29" s="158" t="s">
         <v>338</v>
       </c>
       <c r="I29" s="95"/>
       <c r="J29" s="93" t="s">
         <v>339</v>
       </c>
-      <c r="K29" s="157" t="s">
+      <c r="K29" s="158" t="s">
         <v>340</v>
       </c>
       <c r="L29" s="95"/>
@@ -11018,80 +11017,80 @@
       <c r="N29" s="95"/>
     </row>
     <row r="30" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="164" t="s">
+      <c r="B30" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C30" s="95"/>
-      <c r="D30" s="159" t="s">
+      <c r="D30" s="162" t="s">
         <v>311</v>
       </c>
       <c r="E30" s="95"/>
-      <c r="F30" s="159" t="s">
+      <c r="F30" s="162" t="s">
         <v>341</v>
       </c>
       <c r="G30" s="95"/>
-      <c r="H30" s="159" t="s">
+      <c r="H30" s="162" t="s">
         <v>322</v>
       </c>
       <c r="I30" s="95"/>
       <c r="J30" s="91" t="s">
         <v>342</v>
       </c>
-      <c r="K30" s="159" t="s">
+      <c r="K30" s="162" t="s">
         <v>343</v>
       </c>
       <c r="L30" s="95"/>
       <c r="M30" s="95"/>
       <c r="N30" s="95"/>
     </row>
-    <row r="31" spans="2:14" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="171" t="s">
+    <row r="31" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="163" t="s">
         <v>310</v>
       </c>
       <c r="C31" s="95"/>
-      <c r="D31" s="157" t="s">
+      <c r="D31" s="158" t="s">
         <v>344</v>
       </c>
       <c r="E31" s="95"/>
-      <c r="F31" s="157" t="s">
+      <c r="F31" s="158" t="s">
         <v>345</v>
       </c>
       <c r="G31" s="95"/>
-      <c r="H31" s="157" t="s">
+      <c r="H31" s="158" t="s">
         <v>313</v>
       </c>
       <c r="I31" s="95"/>
       <c r="J31" s="93" t="s">
         <v>346</v>
       </c>
-      <c r="K31" s="157" t="s">
+      <c r="K31" s="158" t="s">
         <v>347</v>
       </c>
       <c r="L31" s="95"/>
       <c r="M31" s="95"/>
       <c r="N31" s="95"/>
     </row>
-    <row r="32" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="164" t="s">
+    <row r="32" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="161" t="s">
         <v>310</v>
       </c>
       <c r="C32" s="95"/>
-      <c r="D32" s="159" t="s">
+      <c r="D32" s="162" t="s">
         <v>344</v>
       </c>
       <c r="E32" s="95"/>
-      <c r="F32" s="159" t="s">
+      <c r="F32" s="162" t="s">
         <v>345</v>
       </c>
       <c r="G32" s="95"/>
-      <c r="H32" s="159" t="s">
+      <c r="H32" s="162" t="s">
         <v>322</v>
       </c>
       <c r="I32" s="95"/>
       <c r="J32" s="91" t="s">
         <v>346</v>
       </c>
-      <c r="K32" s="159" t="s">
+      <c r="K32" s="162" t="s">
         <v>347</v>
       </c>
       <c r="L32" s="95"/>
@@ -11099,7 +11098,7 @@
       <c r="N32" s="95"/>
     </row>
     <row r="40" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="109" t="s">
+      <c r="B40" s="147" t="s">
         <v>348</v>
       </c>
       <c r="C40" s="95"/>
@@ -11116,12 +11115,12 @@
       <c r="N40" s="95"/>
     </row>
     <row r="41" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B41" s="163" t="s">
+      <c r="B41" s="169" t="s">
         <v>349</v>
       </c>
       <c r="C41" s="156"/>
-      <c r="D41" s="97"/>
-      <c r="E41" s="163" t="s">
+      <c r="D41" s="129"/>
+      <c r="E41" s="169" t="s">
         <v>350</v>
       </c>
       <c r="F41" s="156"/>
@@ -11132,15 +11131,15 @@
       <c r="K41" s="156"/>
       <c r="L41" s="156"/>
       <c r="M41" s="156"/>
-      <c r="N41" s="97"/>
+      <c r="N41" s="129"/>
     </row>
     <row r="42" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="160" t="s">
+      <c r="B42" s="157" t="s">
         <v>351</v>
       </c>
       <c r="C42" s="156"/>
-      <c r="D42" s="97"/>
-      <c r="E42" s="161" t="s">
+      <c r="D42" s="129"/>
+      <c r="E42" s="165" t="s">
         <v>352</v>
       </c>
       <c r="F42" s="156"/>
@@ -11151,15 +11150,15 @@
       <c r="K42" s="156"/>
       <c r="L42" s="156"/>
       <c r="M42" s="156"/>
-      <c r="N42" s="97"/>
+      <c r="N42" s="129"/>
     </row>
     <row r="43" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="167" t="s">
+      <c r="B43" s="159" t="s">
         <v>353</v>
       </c>
       <c r="C43" s="156"/>
-      <c r="D43" s="97"/>
-      <c r="E43" s="165" t="s">
+      <c r="D43" s="129"/>
+      <c r="E43" s="160" t="s">
         <v>354</v>
       </c>
       <c r="F43" s="156"/>
@@ -11170,15 +11169,15 @@
       <c r="K43" s="156"/>
       <c r="L43" s="156"/>
       <c r="M43" s="156"/>
-      <c r="N43" s="97"/>
+      <c r="N43" s="129"/>
     </row>
     <row r="44" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="160" t="s">
+      <c r="B44" s="157" t="s">
         <v>355</v>
       </c>
       <c r="C44" s="156"/>
-      <c r="D44" s="97"/>
-      <c r="E44" s="161" t="s">
+      <c r="D44" s="129"/>
+      <c r="E44" s="165" t="s">
         <v>356</v>
       </c>
       <c r="F44" s="156"/>
@@ -11189,15 +11188,15 @@
       <c r="K44" s="156"/>
       <c r="L44" s="156"/>
       <c r="M44" s="156"/>
-      <c r="N44" s="97"/>
+      <c r="N44" s="129"/>
     </row>
     <row r="45" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="167" t="s">
+      <c r="B45" s="159" t="s">
         <v>357</v>
       </c>
       <c r="C45" s="156"/>
-      <c r="D45" s="97"/>
-      <c r="E45" s="165" t="s">
+      <c r="D45" s="129"/>
+      <c r="E45" s="160" t="s">
         <v>354</v>
       </c>
       <c r="F45" s="156"/>
@@ -11208,15 +11207,15 @@
       <c r="K45" s="156"/>
       <c r="L45" s="156"/>
       <c r="M45" s="156"/>
-      <c r="N45" s="97"/>
+      <c r="N45" s="129"/>
     </row>
     <row r="46" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="160" t="s">
+      <c r="B46" s="157" t="s">
         <v>358</v>
       </c>
       <c r="C46" s="156"/>
-      <c r="D46" s="97"/>
-      <c r="E46" s="161" t="s">
+      <c r="D46" s="129"/>
+      <c r="E46" s="165" t="s">
         <v>359</v>
       </c>
       <c r="F46" s="156"/>
@@ -11227,15 +11226,15 @@
       <c r="K46" s="156"/>
       <c r="L46" s="156"/>
       <c r="M46" s="156"/>
-      <c r="N46" s="97"/>
+      <c r="N46" s="129"/>
     </row>
     <row r="47" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="167" t="s">
+      <c r="B47" s="159" t="s">
         <v>360</v>
       </c>
       <c r="C47" s="156"/>
-      <c r="D47" s="97"/>
-      <c r="E47" s="165" t="s">
+      <c r="D47" s="129"/>
+      <c r="E47" s="160" t="s">
         <v>361</v>
       </c>
       <c r="F47" s="156"/>
@@ -11246,15 +11245,15 @@
       <c r="K47" s="156"/>
       <c r="L47" s="156"/>
       <c r="M47" s="156"/>
-      <c r="N47" s="97"/>
+      <c r="N47" s="129"/>
     </row>
     <row r="48" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="160" t="s">
+      <c r="B48" s="157" t="s">
         <v>362</v>
       </c>
       <c r="C48" s="156"/>
-      <c r="D48" s="97"/>
-      <c r="E48" s="161" t="s">
+      <c r="D48" s="129"/>
+      <c r="E48" s="165" t="s">
         <v>363</v>
       </c>
       <c r="F48" s="156"/>
@@ -11265,15 +11264,15 @@
       <c r="K48" s="156"/>
       <c r="L48" s="156"/>
       <c r="M48" s="156"/>
-      <c r="N48" s="97"/>
+      <c r="N48" s="129"/>
     </row>
     <row r="49" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="167" t="s">
+      <c r="B49" s="159" t="s">
         <v>364</v>
       </c>
       <c r="C49" s="156"/>
-      <c r="D49" s="97"/>
-      <c r="E49" s="165" t="s">
+      <c r="D49" s="129"/>
+      <c r="E49" s="160" t="s">
         <v>365</v>
       </c>
       <c r="F49" s="156"/>
@@ -11284,15 +11283,15 @@
       <c r="K49" s="156"/>
       <c r="L49" s="156"/>
       <c r="M49" s="156"/>
-      <c r="N49" s="97"/>
+      <c r="N49" s="129"/>
     </row>
     <row r="50" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="160" t="s">
+      <c r="B50" s="157" t="s">
         <v>366</v>
       </c>
       <c r="C50" s="156"/>
-      <c r="D50" s="97"/>
-      <c r="E50" s="161" t="s">
+      <c r="D50" s="129"/>
+      <c r="E50" s="165" t="s">
         <v>367</v>
       </c>
       <c r="F50" s="156"/>
@@ -11303,10 +11302,10 @@
       <c r="K50" s="156"/>
       <c r="L50" s="156"/>
       <c r="M50" s="156"/>
-      <c r="N50" s="97"/>
+      <c r="N50" s="129"/>
     </row>
     <row r="54" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="94" t="s">
+      <c r="B54" s="152" t="s">
         <v>368</v>
       </c>
       <c r="C54" s="95"/>
@@ -11323,12 +11322,12 @@
       <c r="N54" s="95"/>
     </row>
     <row r="55" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="167" t="s">
+      <c r="B55" s="159" t="s">
         <v>369</v>
       </c>
       <c r="C55" s="156"/>
-      <c r="D55" s="97"/>
-      <c r="E55" s="165" t="s">
+      <c r="D55" s="129"/>
+      <c r="E55" s="160" t="s">
         <v>370</v>
       </c>
       <c r="F55" s="156"/>
@@ -11339,15 +11338,15 @@
       <c r="K55" s="156"/>
       <c r="L55" s="156"/>
       <c r="M55" s="156"/>
-      <c r="N55" s="97"/>
+      <c r="N55" s="129"/>
     </row>
     <row r="56" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="160" t="s">
+      <c r="B56" s="157" t="s">
         <v>371</v>
       </c>
       <c r="C56" s="156"/>
-      <c r="D56" s="97"/>
-      <c r="E56" s="161" t="s">
+      <c r="D56" s="129"/>
+      <c r="E56" s="165" t="s">
         <v>372</v>
       </c>
       <c r="F56" s="156"/>
@@ -11358,15 +11357,15 @@
       <c r="K56" s="156"/>
       <c r="L56" s="156"/>
       <c r="M56" s="156"/>
-      <c r="N56" s="97"/>
+      <c r="N56" s="129"/>
     </row>
     <row r="57" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="167" t="s">
+      <c r="B57" s="159" t="s">
         <v>373</v>
       </c>
       <c r="C57" s="156"/>
-      <c r="D57" s="97"/>
-      <c r="E57" s="165" t="s">
+      <c r="D57" s="129"/>
+      <c r="E57" s="160" t="s">
         <v>374</v>
       </c>
       <c r="F57" s="156"/>
@@ -11377,15 +11376,15 @@
       <c r="K57" s="156"/>
       <c r="L57" s="156"/>
       <c r="M57" s="156"/>
-      <c r="N57" s="97"/>
+      <c r="N57" s="129"/>
     </row>
     <row r="58" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="160" t="s">
+      <c r="B58" s="157" t="s">
         <v>375</v>
       </c>
       <c r="C58" s="156"/>
-      <c r="D58" s="97"/>
-      <c r="E58" s="161" t="s">
+      <c r="D58" s="129"/>
+      <c r="E58" s="165" t="s">
         <v>376</v>
       </c>
       <c r="F58" s="156"/>
@@ -11396,15 +11395,15 @@
       <c r="K58" s="156"/>
       <c r="L58" s="156"/>
       <c r="M58" s="156"/>
-      <c r="N58" s="97"/>
+      <c r="N58" s="129"/>
     </row>
     <row r="59" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="167" t="s">
+      <c r="B59" s="159" t="s">
         <v>377</v>
       </c>
       <c r="C59" s="156"/>
-      <c r="D59" s="97"/>
-      <c r="E59" s="165" t="s">
+      <c r="D59" s="129"/>
+      <c r="E59" s="160" t="s">
         <v>378</v>
       </c>
       <c r="F59" s="156"/>
@@ -11415,15 +11414,15 @@
       <c r="K59" s="156"/>
       <c r="L59" s="156"/>
       <c r="M59" s="156"/>
-      <c r="N59" s="97"/>
+      <c r="N59" s="129"/>
     </row>
     <row r="60" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B60" s="160" t="s">
+      <c r="B60" s="157" t="s">
         <v>379</v>
       </c>
       <c r="C60" s="156"/>
-      <c r="D60" s="97"/>
-      <c r="E60" s="161" t="s">
+      <c r="D60" s="129"/>
+      <c r="E60" s="165" t="s">
         <v>380</v>
       </c>
       <c r="F60" s="156"/>
@@ -11434,15 +11433,15 @@
       <c r="K60" s="156"/>
       <c r="L60" s="156"/>
       <c r="M60" s="156"/>
-      <c r="N60" s="97"/>
+      <c r="N60" s="129"/>
     </row>
     <row r="61" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="167" t="s">
+      <c r="B61" s="159" t="s">
         <v>381</v>
       </c>
       <c r="C61" s="156"/>
-      <c r="D61" s="97"/>
-      <c r="E61" s="165" t="s">
+      <c r="D61" s="129"/>
+      <c r="E61" s="160" t="s">
         <v>382</v>
       </c>
       <c r="F61" s="156"/>
@@ -11453,15 +11452,15 @@
       <c r="K61" s="156"/>
       <c r="L61" s="156"/>
       <c r="M61" s="156"/>
-      <c r="N61" s="97"/>
+      <c r="N61" s="129"/>
     </row>
     <row r="62" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="160" t="s">
+      <c r="B62" s="157" t="s">
         <v>383</v>
       </c>
       <c r="C62" s="156"/>
-      <c r="D62" s="97"/>
-      <c r="E62" s="161" t="s">
+      <c r="D62" s="129"/>
+      <c r="E62" s="165" t="s">
         <v>384</v>
       </c>
       <c r="F62" s="156"/>
@@ -11472,15 +11471,15 @@
       <c r="K62" s="156"/>
       <c r="L62" s="156"/>
       <c r="M62" s="156"/>
-      <c r="N62" s="97"/>
+      <c r="N62" s="129"/>
     </row>
     <row r="63" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="162" t="s">
+      <c r="B63" s="170" t="s">
         <v>385</v>
       </c>
       <c r="C63" s="156"/>
-      <c r="D63" s="97"/>
-      <c r="E63" s="162" t="s">
+      <c r="D63" s="129"/>
+      <c r="E63" s="170" t="s">
         <v>386</v>
       </c>
       <c r="F63" s="156"/>
@@ -11491,20 +11490,96 @@
       <c r="K63" s="156"/>
       <c r="L63" s="156"/>
       <c r="M63" s="156"/>
-      <c r="N63" s="97"/>
+      <c r="N63" s="129"/>
     </row>
   </sheetData>
   <mergeCells count="130">
-    <mergeCell ref="K24:N24"/>
-    <mergeCell ref="E41:N41"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B54:N54"/>
-    <mergeCell ref="E55:N55"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="E48:N48"/>
-    <mergeCell ref="K20:N20"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="K22:N22"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="E62:N62"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="K29:N29"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="E49:N49"/>
+    <mergeCell ref="K23:N23"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="E50:N50"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="K32:N32"/>
+    <mergeCell ref="E63:N63"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E60:N60"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E45:N45"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B40:N40"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="E47:N47"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="E56:N56"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E43:N43"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="K21:N21"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E15:H15"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B19:N19"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E42:N42"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="K26:N26"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="E44:N44"/>
@@ -11529,102 +11604,26 @@
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="K21:N21"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E15:H15"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B19:N19"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E42:N42"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:N57"/>
     <mergeCell ref="F25:G25"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B31:C31"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="E63:N63"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="E60:N60"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="E45:N45"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B40:N40"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="E62:N62"/>
-    <mergeCell ref="B20:J20"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="E49:N49"/>
-    <mergeCell ref="K23:N23"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="E50:N50"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="K22:N22"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="E47:N47"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="E56:N56"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E43:N43"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="E57:N57"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="E58:N58"/>
+    <mergeCell ref="K24:N24"/>
+    <mergeCell ref="E41:N41"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B54:N54"/>
+    <mergeCell ref="E55:N55"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="E48:N48"/>
+    <mergeCell ref="K20:N20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>